<commit_message>
v105: map 100% to 20 points on the score scale.
0 points stay 0% and 10 points stay 50%. The live rules workbook is
regenerated with the new high end.
</commit_message>
<xml_diff>
--- a/현재_규칙.xlsx
+++ b/현재_규칙.xlsx
@@ -558,7 +558,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>지금 적용 규칙 · 앱 v104</t>
+          <t>지금 적용 규칙 · 앱 v105</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2. 합산 점수를 %로 바꿉니다. 0점 이하=0%, 10점=50%, 19점 이상=100%.</t>
+          <t>2. 합산 점수를 %로 바꿉니다. 0점 이하=0%, 10점=50%, 20점 이상=100%.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>점수를 %로 바꾸는 법: 0점 이하=0%, 10점(기본)=50%, 19점 이상=100%.</t>
+          <t>점수를 %로 바꾸는 법: 0점 이하=0%, 10점(기본)=50%, 20점 이상=100%.</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1831,7 +1831,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="18">
-        <f>ROUND(IF(A2&lt;=0,0,IF(A2&gt;=19,100,IF(A2&lt;=10,(A2-0)/10*50,50+(A2-10)/9*50))),0)</f>
+        <f>ROUND(IF(A2&lt;=0,0,IF(A2&gt;=20,100,IF(A2&lt;=10,(A2-0)/10*50,50+(A2-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -1858,7 +1858,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="18">
-        <f>ROUND(IF(A3&lt;=0,0,IF(A3&gt;=19,100,IF(A3&lt;=10,(A3-0)/10*50,50+(A3-10)/9*50))),0)</f>
+        <f>ROUND(IF(A3&lt;=0,0,IF(A3&gt;=20,100,IF(A3&lt;=10,(A3-0)/10*50,50+(A3-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -1885,7 +1885,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="18">
-        <f>ROUND(IF(A4&lt;=0,0,IF(A4&gt;=19,100,IF(A4&lt;=10,(A4-0)/10*50,50+(A4-10)/9*50))),0)</f>
+        <f>ROUND(IF(A4&lt;=0,0,IF(A4&gt;=20,100,IF(A4&lt;=10,(A4-0)/10*50,50+(A4-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1912,7 +1912,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="18">
-        <f>ROUND(IF(A5&lt;=0,0,IF(A5&gt;=19,100,IF(A5&lt;=10,(A5-0)/10*50,50+(A5-10)/9*50))),0)</f>
+        <f>ROUND(IF(A5&lt;=0,0,IF(A5&gt;=20,100,IF(A5&lt;=10,(A5-0)/10*50,50+(A5-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="18">
-        <f>ROUND(IF(A6&lt;=0,0,IF(A6&gt;=19,100,IF(A6&lt;=10,(A6-0)/10*50,50+(A6-10)/9*50))),0)</f>
+        <f>ROUND(IF(A6&lt;=0,0,IF(A6&gt;=20,100,IF(A6&lt;=10,(A6-0)/10*50,50+(A6-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1966,7 +1966,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="18">
-        <f>ROUND(IF(A7&lt;=0,0,IF(A7&gt;=19,100,IF(A7&lt;=10,(A7-0)/10*50,50+(A7-10)/9*50))),0)</f>
+        <f>ROUND(IF(A7&lt;=0,0,IF(A7&gt;=20,100,IF(A7&lt;=10,(A7-0)/10*50,50+(A7-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1993,7 +1993,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="18">
-        <f>ROUND(IF(A8&lt;=0,0,IF(A8&gt;=19,100,IF(A8&lt;=10,(A8-0)/10*50,50+(A8-10)/9*50))),0)</f>
+        <f>ROUND(IF(A8&lt;=0,0,IF(A8&gt;=20,100,IF(A8&lt;=10,(A8-0)/10*50,50+(A8-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -2020,7 +2020,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="18">
-        <f>ROUND(IF(A9&lt;=0,0,IF(A9&gt;=19,100,IF(A9&lt;=10,(A9-0)/10*50,50+(A9-10)/9*50))),0)</f>
+        <f>ROUND(IF(A9&lt;=0,0,IF(A9&gt;=20,100,IF(A9&lt;=10,(A9-0)/10*50,50+(A9-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -2047,7 +2047,7 @@
         <v>25</v>
       </c>
       <c r="C10" s="18">
-        <f>ROUND(IF(A10&lt;=0,0,IF(A10&gt;=19,100,IF(A10&lt;=10,(A10-0)/10*50,50+(A10-10)/9*50))),0)</f>
+        <f>ROUND(IF(A10&lt;=0,0,IF(A10&gt;=20,100,IF(A10&lt;=10,(A10-0)/10*50,50+(A10-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -2074,7 +2074,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="18">
-        <f>ROUND(IF(A11&lt;=0,0,IF(A11&gt;=19,100,IF(A11&lt;=10,(A11-0)/10*50,50+(A11-10)/9*50))),0)</f>
+        <f>ROUND(IF(A11&lt;=0,0,IF(A11&gt;=20,100,IF(A11&lt;=10,(A11-0)/10*50,50+(A11-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -2101,7 +2101,7 @@
         <v>35</v>
       </c>
       <c r="C12" s="18">
-        <f>ROUND(IF(A12&lt;=0,0,IF(A12&gt;=19,100,IF(A12&lt;=10,(A12-0)/10*50,50+(A12-10)/9*50))),0)</f>
+        <f>ROUND(IF(A12&lt;=0,0,IF(A12&gt;=20,100,IF(A12&lt;=10,(A12-0)/10*50,50+(A12-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2128,7 +2128,7 @@
         <v>40</v>
       </c>
       <c r="C13" s="18">
-        <f>ROUND(IF(A13&lt;=0,0,IF(A13&gt;=19,100,IF(A13&lt;=10,(A13-0)/10*50,50+(A13-10)/9*50))),0)</f>
+        <f>ROUND(IF(A13&lt;=0,0,IF(A13&gt;=20,100,IF(A13&lt;=10,(A13-0)/10*50,50+(A13-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -2155,7 +2155,7 @@
         <v>45</v>
       </c>
       <c r="C14" s="18">
-        <f>ROUND(IF(A14&lt;=0,0,IF(A14&gt;=19,100,IF(A14&lt;=10,(A14-0)/10*50,50+(A14-10)/9*50))),0)</f>
+        <f>ROUND(IF(A14&lt;=0,0,IF(A14&gt;=20,100,IF(A14&lt;=10,(A14-0)/10*50,50+(A14-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2182,7 +2182,7 @@
         <v>50</v>
       </c>
       <c r="C15" s="18">
-        <f>ROUND(IF(A15&lt;=0,0,IF(A15&gt;=19,100,IF(A15&lt;=10,(A15-0)/10*50,50+(A15-10)/9*50))),0)</f>
+        <f>ROUND(IF(A15&lt;=0,0,IF(A15&gt;=20,100,IF(A15&lt;=10,(A15-0)/10*50,50+(A15-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -2206,15 +2206,15 @@
         <v>11</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C16" s="18">
-        <f>ROUND(IF(A16&lt;=0,0,IF(A16&gt;=19,100,IF(A16&lt;=10,(A16-0)/10*50,50+(A16-10)/9*50))),0)</f>
+        <f>ROUND(IF(A16&lt;=0,0,IF(A16&gt;=20,100,IF(A16&lt;=10,(A16-0)/10*50,50+(A16-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>50+(11-10)/9×50 = 55.556 → 56%</t>
+          <t>50+(11-10)/10×50 = 55.000 → 55%</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -2233,15 +2233,15 @@
         <v>12</v>
       </c>
       <c r="B17" s="18" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="18">
-        <f>ROUND(IF(A17&lt;=0,0,IF(A17&gt;=19,100,IF(A17&lt;=10,(A17-0)/10*50,50+(A17-10)/9*50))),0)</f>
+        <f>ROUND(IF(A17&lt;=0,0,IF(A17&gt;=20,100,IF(A17&lt;=10,(A17-0)/10*50,50+(A17-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>50+(12-10)/9×50 = 61.111 → 61%</t>
+          <t>50+(12-10)/10×50 = 60.000 → 60%</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
@@ -2260,15 +2260,15 @@
         <v>13</v>
       </c>
       <c r="B18" s="18" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C18" s="18">
-        <f>ROUND(IF(A18&lt;=0,0,IF(A18&gt;=19,100,IF(A18&lt;=10,(A18-0)/10*50,50+(A18-10)/9*50))),0)</f>
+        <f>ROUND(IF(A18&lt;=0,0,IF(A18&gt;=20,100,IF(A18&lt;=10,(A18-0)/10*50,50+(A18-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>50+(13-10)/9×50 = 66.667 → 67%</t>
+          <t>50+(13-10)/10×50 = 65.000 → 65%</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -2287,15 +2287,15 @@
         <v>14</v>
       </c>
       <c r="B19" s="18" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C19" s="18">
-        <f>ROUND(IF(A19&lt;=0,0,IF(A19&gt;=19,100,IF(A19&lt;=10,(A19-0)/10*50,50+(A19-10)/9*50))),0)</f>
+        <f>ROUND(IF(A19&lt;=0,0,IF(A19&gt;=20,100,IF(A19&lt;=10,(A19-0)/10*50,50+(A19-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>50+(14-10)/9×50 = 72.222 → 72%</t>
+          <t>50+(14-10)/10×50 = 70.000 → 70%</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
@@ -2314,15 +2314,15 @@
         <v>15</v>
       </c>
       <c r="B20" s="18" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C20" s="18">
-        <f>ROUND(IF(A20&lt;=0,0,IF(A20&gt;=19,100,IF(A20&lt;=10,(A20-0)/10*50,50+(A20-10)/9*50))),0)</f>
+        <f>ROUND(IF(A20&lt;=0,0,IF(A20&gt;=20,100,IF(A20&lt;=10,(A20-0)/10*50,50+(A20-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>50+(15-10)/9×50 = 77.778 → 78%</t>
+          <t>50+(15-10)/10×50 = 75.000 → 75%</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -2341,15 +2341,15 @@
         <v>16</v>
       </c>
       <c r="B21" s="18" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C21" s="18">
-        <f>ROUND(IF(A21&lt;=0,0,IF(A21&gt;=19,100,IF(A21&lt;=10,(A21-0)/10*50,50+(A21-10)/9*50))),0)</f>
+        <f>ROUND(IF(A21&lt;=0,0,IF(A21&gt;=20,100,IF(A21&lt;=10,(A21-0)/10*50,50+(A21-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>50+(16-10)/9×50 = 83.333 → 83%</t>
+          <t>50+(16-10)/10×50 = 80.000 → 80%</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -2368,15 +2368,15 @@
         <v>17</v>
       </c>
       <c r="B22" s="18" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C22" s="18">
-        <f>ROUND(IF(A22&lt;=0,0,IF(A22&gt;=19,100,IF(A22&lt;=10,(A22-0)/10*50,50+(A22-10)/9*50))),0)</f>
+        <f>ROUND(IF(A22&lt;=0,0,IF(A22&gt;=20,100,IF(A22&lt;=10,(A22-0)/10*50,50+(A22-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>50+(17-10)/9×50 = 88.889 → 89%</t>
+          <t>50+(17-10)/10×50 = 85.000 → 85%</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -2395,15 +2395,15 @@
         <v>18</v>
       </c>
       <c r="B23" s="18" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C23" s="18">
-        <f>ROUND(IF(A23&lt;=0,0,IF(A23&gt;=19,100,IF(A23&lt;=10,(A23-0)/10*50,50+(A23-10)/9*50))),0)</f>
+        <f>ROUND(IF(A23&lt;=0,0,IF(A23&gt;=20,100,IF(A23&lt;=10,(A23-0)/10*50,50+(A23-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>50+(18-10)/9×50 = 94.444 → 94%</t>
+          <t>50+(18-10)/10×50 = 90.000 → 90%</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
@@ -2422,15 +2422,15 @@
         <v>19</v>
       </c>
       <c r="B24" s="18" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C24" s="18">
-        <f>ROUND(IF(A24&lt;=0,0,IF(A24&gt;=19,100,IF(A24&lt;=10,(A24-0)/10*50,50+(A24-10)/9*50))),0)</f>
+        <f>ROUND(IF(A24&lt;=0,0,IF(A24&gt;=20,100,IF(A24&lt;=10,(A24-0)/10*50,50+(A24-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>50+(19-10)/9×50 = 100.000 → 100%</t>
+          <t>50+(19-10)/10×50 = 95.000 → 95%</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -2452,12 +2452,12 @@
         <v>100</v>
       </c>
       <c r="C25" s="18">
-        <f>ROUND(IF(A25&lt;=0,0,IF(A25&gt;=19,100,IF(A25&lt;=10,(A25-0)/10*50,50+(A25-10)/9*50))),0)</f>
+        <f>ROUND(IF(A25&lt;=0,0,IF(A25&gt;=20,100,IF(A25&lt;=10,(A25-0)/10*50,50+(A25-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>20점 → 19점으로 보고 100%</t>
+          <t>50+(20-10)/10×50 = 100.000 → 100%</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -2479,12 +2479,12 @@
         <v>100</v>
       </c>
       <c r="C26" s="18">
-        <f>ROUND(IF(A26&lt;=0,0,IF(A26&gt;=19,100,IF(A26&lt;=10,(A26-0)/10*50,50+(A26-10)/9*50))),0)</f>
+        <f>ROUND(IF(A26&lt;=0,0,IF(A26&gt;=20,100,IF(A26&lt;=10,(A26-0)/10*50,50+(A26-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>21점 → 19점으로 보고 100%</t>
+          <t>21점 → 20점으로 보고 100%</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -2506,12 +2506,12 @@
         <v>100</v>
       </c>
       <c r="C27" s="18">
-        <f>ROUND(IF(A27&lt;=0,0,IF(A27&gt;=19,100,IF(A27&lt;=10,(A27-0)/10*50,50+(A27-10)/9*50))),0)</f>
+        <f>ROUND(IF(A27&lt;=0,0,IF(A27&gt;=20,100,IF(A27&lt;=10,(A27-0)/10*50,50+(A27-10)/10*50))),0)</f>
         <v/>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>22점 → 19점으로 보고 100%</t>
+          <t>22점 → 20점으로 보고 100%</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
@@ -2520,6 +2520,33 @@
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>강한 매수</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="18">
+        <f>ROUND(IF(A28&lt;=0,0,IF(A28&gt;=20,100,IF(A28&lt;=10,(A28-0)/10*50,50+(A28-10)/10*50))),0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>23점 → 20점으로 보고 100%</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>강한 매수</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
         <is>
           <t>강한 매수</t>
         </is>
@@ -2576,7 +2603,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  상한 HI = 19점  →  100%</t>
+          <t xml:space="preserve">  상한 HI = 20점  →  100%</t>
         </is>
       </c>
     </row>
@@ -2607,14 +2634,14 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  10 &lt; s &lt; 19  →  ROUND( 50 + (s-10)/9 × 50 )</t>
+          <t xml:space="preserve">  10 &lt; s &lt; 20  →  ROUND( 50 + (s-10)/10 × 50 )</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  s ≥ 19  →  100%</t>
+          <t xml:space="preserve">  s ≥ 20  →  100%</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2658,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =ROUND(IF(A2&lt;=0,0,IF(A2&gt;=19,100,IF(A2&lt;=10,(A2-0)/10*50,50+(A2-10)/9*50))),0)</t>
+          <t xml:space="preserve">  =ROUND(IF(A2&lt;=0,0,IF(A2&gt;=20,100,IF(A2&lt;=10,(A2-0)/10*50,50+(A2-10)/10*50))),0)</t>
         </is>
       </c>
     </row>

</xml_diff>